<commit_message>
Refactor main application structure by consolidating API endpoints into routers for aircraft, APC, catalog, and PD. Remove deprecated endpoint definitions and streamline the FastAPI application setup. Update PD store service with new methods for handling issue versions and attempts, and enhance validation rules for source files. Update frontend help documentation to reflect changes in file handling and validation requirements.
</commit_message>
<xml_diff>
--- a/Test/pd/fail-issue-name.xlsx
+++ b/Test/pd/fail-issue-name.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PD" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PD-SUMMARY" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M6"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -478,11 +478,6 @@
           <t>01.00</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>Version</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -545,7 +540,6 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -608,7 +602,6 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -671,7 +664,6 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -722,7 +714,6 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -785,7 +776,6 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>